<commit_message>
Deliver DEV211 UAT210 remediation
</commit_message>
<xml_diff>
--- a/public/templates/purchased-customer-import-template.xlsx
+++ b/public/templates/purchased-customer-import-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rfa68a984f5da4922"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch" sheetId="2" r:id="Rcbad895f9f2141b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="3" r:id="R063b7748a46342e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rf7d44dbeade64ef3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch" sheetId="2" r:id="Rd10a7ae9daec4c4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="3" r:id="R28218c22f5594148"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -323,7 +323,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>NYSA Bulk Customer Import Template</x:v>
+        <x:v>NYSA Bulk Customer Upload Template</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>

</xml_diff>